<commit_message>
personal: some additions to my research
</commit_message>
<xml_diff>
--- a/personal_projects/productivity_logs/logs.xlsx
+++ b/personal_projects/productivity_logs/logs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bagim\Desktop\My_projects\personal_projects\productivity_logs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B12BCE6-EBF8-4654-9A2D-1B59C3DF2A14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{950F79F7-35C0-44E7-9EEB-CE16FF3389E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -537,13 +537,11 @@
         <v>45926</v>
       </c>
       <c r="B23">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" s="1">
-        <v>45927</v>
-      </c>
+      <c r="A24" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>